<commit_message>
Remove every duplicate selector
</commit_message>
<xml_diff>
--- a/excel_sheets/November_2026.xlsx
+++ b/excel_sheets/November_2026.xlsx
@@ -552,14 +552,14 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" s="4" t="n">
-        <v>1111</v>
+        <v>1111888</v>
       </c>
       <c r="G3" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" s="4" t="n">
-        <v>112222</v>
+        <v>1222999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>